<commit_message>
Correct Gandul 2,4 against Gambar 2.12
Three faults found by comparing the render with the book figure:

ASARI and CSW were modelled as busbars on Tier-3 and Tier-4. Gambar 2.12
draws both as dashed arrows hanging off a busbar, the same symbol as
SWGAN and CRNDE, so they are bays: ASARI on KMANG and CSW on SAMBAS.
Modelling them as busbars invented a fourth tier the figure does not
have, and left them looking like network nodes rather than loads.

Gandul - Pondok Indah was written as SUTT. It is a cable like
Gandul - Kemang, which risk 1 names explicitly as SKTT. The parser reads
the circuit type from the penghantar name, so the name now says SKTT.

The sheet drops from 4 tiers to 3 and from 5 ruas to 3, which is what
the figure shows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/ss_gndul24_ingest.xlsx
+++ b/samples/ss_gndul24_ingest.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -906,12 +906,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Asari</t>
+          <t>Sambas (aset milik KTT)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ASARI</t>
+          <t>SAMBAS</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -932,7 +932,11 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>aset milik KTT</t>
+        </is>
+      </c>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
@@ -952,120 +956,6 @@
         </is>
       </c>
       <c r="S7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Sambas (aset milik KTT)</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>SAMBAS</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Busbar GI</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>2</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>150 kV</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>aset milik KTT</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>Beroperasi</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>DKI Jakarta</t>
-        </is>
-      </c>
-      <c r="S8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CSW (aset milik KTT)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>CSW</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Busbar GI</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>150 kV</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>aset milik KTT</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>Beroperasi</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>DKI Jakarta</t>
-        </is>
-      </c>
-      <c r="S9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1078,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1175,7 +1065,7 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>SUTT Gandul - Pondok Indah</t>
+          <t>SKTT 150 kV Gandul - Pondok Indah</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1297,17 +1187,17 @@
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SUTT Kemang - Asari</t>
+          <t>SUTT Pondok Indah - Sambas (aset milik KTT)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>KMANG</t>
+          <t>PNDAH</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ASARI</t>
+          <t>SAMBAS</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1348,124 +1238,6 @@
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>SUTT Pondok Indah - Sambas (aset milik KTT)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>PNDAH</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>SAMBAS</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>150 kV</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>Beroperasi</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>DKI Jakarta</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>2</v>
-      </c>
-      <c r="O5" t="n">
-        <v>3</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Tidak</t>
-        </is>
-      </c>
-      <c r="Q5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>SUTT Sambas - CSW (aset milik KTT)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>SAMBAS</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>CSW</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>150 kV</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Beroperasi</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>DKI Jakarta</t>
-        </is>
-      </c>
-      <c r="N6" t="n">
-        <v>3</v>
-      </c>
-      <c r="O6" t="n">
-        <v>4</v>
-      </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>Tidak</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1478,7 +1250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1597,6 +1369,76 @@
       </c>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ASARI</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Asari</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>KMANG</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CSW</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>CSW (aset milik KTT)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SAMBAS</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>150 kV</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Beroperasi</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>